<commit_message>
Add ONS time series codes and HR1 redundancy notifications
- Added new column E (ONS Time Series Code) with A01 dataset identifier
  codes for each variable (e.g. MGRZ, MGSC, LF24, BEAO, KAB9, AP2Y)
- Added HR1 redundancy notifications (Insolvency Service) from Top Ten Stats

https://claude.ai/code/session_01Uxu3nd6u3avwpdkB8AAoBh
</commit_message>
<xml_diff>
--- a/TLFS Variable Prioritisation Mapping.xlsx
+++ b/TLFS Variable Prioritisation Mapping.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="15.5703125" customWidth="1" min="1" max="1"/>
@@ -477,6 +477,11 @@
           <t>Core or Plus (to be completed)</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ONS Time Series Code</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="43.5" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
@@ -561,6 +566,11 @@
           <t>ILODEFR</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>MGRZ</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -573,6 +583,11 @@
           <t>ILODEFR</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LF24</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -585,6 +600,11 @@
           <t>ILODEFR</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>MGSC</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -597,6 +617,11 @@
           <t>ILODEFR</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>MGSX</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -609,6 +634,11 @@
           <t>ILODEFR</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LF2M</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -621,6 +651,11 @@
           <t>ILODEFR</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LF2S</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -633,6 +668,11 @@
           <t>INECAC05</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LF69</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -645,6 +685,11 @@
           <t>INECAC05</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LF63</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -657,6 +702,11 @@
           <t>INECAC05</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LF65</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -669,6 +719,11 @@
           <t>INECAC05</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LF6B</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -681,6 +736,11 @@
           <t>REDUND</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>BEAO (level) ; BEIR (rate)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -693,6 +753,11 @@
           <t>INECAC05 ; AGE</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>YBVN (level) ; YBVQ (rate)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -705,6 +770,11 @@
           <t>INECAC05 ; AGE</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LF2A (level) ; LF2W (rate)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -765,6 +835,11 @@
           <t>N/A - AWE</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>KAB9 (level) ; KAC3 (3m avg %)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -777,6 +852,11 @@
           <t>N/A - AWE</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>KAI7 (level) ; KAI9 (3m avg %)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -789,6 +869,11 @@
           <t>N/A - AWE</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>A3WX (total) ; A2FC (regular)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -801,6 +886,11 @@
           <t>N/A - Vacancy Survey</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>AP2Y</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -813,6 +903,11 @@
           <t>N/A - Labour Disputes Inquiry</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>BBFW</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -825,6 +920,11 @@
           <t>N/A - Employer surveys / LFS / admin</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>DYDC</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -835,6 +935,18 @@
       <c r="B31" t="inlineStr">
         <is>
           <t>GRSSWK</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>HR1 redundancy notifications (Insolvency Service)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>N/A - Insolvency Service admin data</t>
         </is>
       </c>
     </row>

</xml_diff>